<commit_message>
Agrega slug a todos los productos
</commit_message>
<xml_diff>
--- a/public/Plantilla_Quimica_Bethel_2.0.xlsx
+++ b/public/Plantilla_Quimica_Bethel_2.0.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\facun\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{75E5983A-D124-4D35-9A2C-CED096121448}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A584AA08-478B-4A55-966A-14E06A3B5FA0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="19440" windowHeight="14880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4245" uniqueCount="1537">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4378" uniqueCount="1538">
   <si>
     <t>ID</t>
   </si>
@@ -4343,24 +4343,6 @@
     <t>SHA001</t>
   </si>
   <si>
-    <t>SHA001.jpg</t>
-  </si>
-  <si>
-    <t>SHA002.jpg</t>
-  </si>
-  <si>
-    <t>SHA003.jpg</t>
-  </si>
-  <si>
-    <t>SHA004.jpg</t>
-  </si>
-  <si>
-    <t>SHA005.jpg</t>
-  </si>
-  <si>
-    <t>SHA006.jpg</t>
-  </si>
-  <si>
     <t>Shampoo para manos por 5 litros</t>
   </si>
   <si>
@@ -4650,6 +4632,27 @@
   </si>
   <si>
     <t>PROM003.png</t>
+  </si>
+  <si>
+    <t>SHA001.png</t>
+  </si>
+  <si>
+    <t>SHA002.png</t>
+  </si>
+  <si>
+    <t>SHA003.png</t>
+  </si>
+  <si>
+    <t>SHA004.png</t>
+  </si>
+  <si>
+    <t>SHA005.png</t>
+  </si>
+  <si>
+    <t>SHA006.png</t>
+  </si>
+  <si>
+    <t>SLUG</t>
   </si>
 </sst>
 </file>
@@ -5009,14 +5012,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:P1001"/>
+  <dimension ref="A1:Q1001"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="6" max="6" width="26.140625" customWidth="1"/>
     <col min="7" max="7" width="23" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -5065,8 +5068,11 @@
       <c r="P1" s="1" t="s">
         <v>1357</v>
       </c>
-    </row>
-    <row r="2" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="Q1" s="1" t="s">
+        <v>1537</v>
+      </c>
+    </row>
+    <row r="2" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>15</v>
       </c>
@@ -5092,14 +5098,14 @@
         <v>1078</v>
       </c>
       <c r="J2">
-        <v>2300</v>
+        <v>3300</v>
       </c>
       <c r="K2">
-        <v>4</v>
+        <v>0.5</v>
       </c>
       <c r="L2">
         <f t="shared" ref="L2:L65" si="0">IF(J2="","",J2*(1+K2))</f>
-        <v>11500</v>
+        <v>4950</v>
       </c>
       <c r="M2" t="s">
         <v>16</v>
@@ -5110,8 +5116,11 @@
       <c r="P2" t="s">
         <v>1359</v>
       </c>
-    </row>
-    <row r="3" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="Q2" t="s">
+        <v>1077</v>
+      </c>
+    </row>
+    <row r="3" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>17</v>
       </c>
@@ -5155,8 +5164,11 @@
       <c r="P3" t="s">
         <v>1359</v>
       </c>
-    </row>
-    <row r="4" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="Q3" t="s">
+        <v>1079</v>
+      </c>
+    </row>
+    <row r="4" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>18</v>
       </c>
@@ -5200,8 +5212,11 @@
       <c r="P4" t="s">
         <v>1359</v>
       </c>
-    </row>
-    <row r="5" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="Q4" t="s">
+        <v>1084</v>
+      </c>
+    </row>
+    <row r="5" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>19</v>
       </c>
@@ -5245,8 +5260,11 @@
       <c r="P5" t="s">
         <v>1359</v>
       </c>
-    </row>
-    <row r="6" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="Q5" t="s">
+        <v>1085</v>
+      </c>
+    </row>
+    <row r="6" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>20</v>
       </c>
@@ -5293,8 +5311,11 @@
       <c r="P6" t="s">
         <v>1359</v>
       </c>
-    </row>
-    <row r="7" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="Q6" t="s">
+        <v>1092</v>
+      </c>
+    </row>
+    <row r="7" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>21</v>
       </c>
@@ -5341,8 +5362,11 @@
       <c r="P7" t="s">
         <v>1359</v>
       </c>
-    </row>
-    <row r="8" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="Q7" t="s">
+        <v>1093</v>
+      </c>
+    </row>
+    <row r="8" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>22</v>
       </c>
@@ -5386,8 +5410,11 @@
       <c r="P8" t="s">
         <v>1359</v>
       </c>
-    </row>
-    <row r="9" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="Q8" t="s">
+        <v>1100</v>
+      </c>
+    </row>
+    <row r="9" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>23</v>
       </c>
@@ -5434,8 +5461,11 @@
       <c r="P9" t="s">
         <v>1359</v>
       </c>
-    </row>
-    <row r="10" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="Q9" t="s">
+        <v>1106</v>
+      </c>
+    </row>
+    <row r="10" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>24</v>
       </c>
@@ -5482,8 +5512,11 @@
       <c r="P10" t="s">
         <v>1359</v>
       </c>
-    </row>
-    <row r="11" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="Q10" t="s">
+        <v>1112</v>
+      </c>
+    </row>
+    <row r="11" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>25</v>
       </c>
@@ -5527,8 +5560,11 @@
       <c r="P11" t="s">
         <v>1359</v>
       </c>
-    </row>
-    <row r="12" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="Q11" t="s">
+        <v>1117</v>
+      </c>
+    </row>
+    <row r="12" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>26</v>
       </c>
@@ -5572,8 +5608,11 @@
       <c r="P12" t="s">
         <v>1359</v>
       </c>
-    </row>
-    <row r="13" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="Q12" t="s">
+        <v>1118</v>
+      </c>
+    </row>
+    <row r="13" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>27</v>
       </c>
@@ -5617,8 +5656,11 @@
       <c r="P13" t="s">
         <v>1359</v>
       </c>
-    </row>
-    <row r="14" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="Q13" t="s">
+        <v>1119</v>
+      </c>
+    </row>
+    <row r="14" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>28</v>
       </c>
@@ -5662,8 +5704,11 @@
       <c r="P14" t="s">
         <v>1359</v>
       </c>
-    </row>
-    <row r="15" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="Q14" t="s">
+        <v>1120</v>
+      </c>
+    </row>
+    <row r="15" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>29</v>
       </c>
@@ -5707,8 +5752,11 @@
       <c r="P15" t="s">
         <v>1359</v>
       </c>
-    </row>
-    <row r="16" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="Q15" t="s">
+        <v>1121</v>
+      </c>
+    </row>
+    <row r="16" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>30</v>
       </c>
@@ -5752,8 +5800,11 @@
       <c r="P16" t="s">
         <v>1359</v>
       </c>
-    </row>
-    <row r="17" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="Q16" t="s">
+        <v>1139</v>
+      </c>
+    </row>
+    <row r="17" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>31</v>
       </c>
@@ -5797,8 +5848,11 @@
       <c r="P17" t="s">
         <v>1359</v>
       </c>
-    </row>
-    <row r="18" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="Q17" t="s">
+        <v>1140</v>
+      </c>
+    </row>
+    <row r="18" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>32</v>
       </c>
@@ -5842,8 +5896,11 @@
       <c r="P18" t="s">
         <v>1359</v>
       </c>
-    </row>
-    <row r="19" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="Q18" t="s">
+        <v>1141</v>
+      </c>
+    </row>
+    <row r="19" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>33</v>
       </c>
@@ -5887,8 +5944,11 @@
       <c r="P19" t="s">
         <v>1359</v>
       </c>
-    </row>
-    <row r="20" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="Q19" t="s">
+        <v>1142</v>
+      </c>
+    </row>
+    <row r="20" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>34</v>
       </c>
@@ -5932,8 +5992,11 @@
       <c r="P20" t="s">
         <v>1359</v>
       </c>
-    </row>
-    <row r="21" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="Q20" t="s">
+        <v>1143</v>
+      </c>
+    </row>
+    <row r="21" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>35</v>
       </c>
@@ -5977,8 +6040,11 @@
       <c r="P21" t="s">
         <v>1359</v>
       </c>
-    </row>
-    <row r="22" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="Q21" t="s">
+        <v>1144</v>
+      </c>
+    </row>
+    <row r="22" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>36</v>
       </c>
@@ -6022,8 +6088,11 @@
       <c r="P22" t="s">
         <v>1359</v>
       </c>
-    </row>
-    <row r="23" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="Q22" t="s">
+        <v>1145</v>
+      </c>
+    </row>
+    <row r="23" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>37</v>
       </c>
@@ -6067,8 +6136,11 @@
       <c r="P23" t="s">
         <v>1359</v>
       </c>
-    </row>
-    <row r="24" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="Q23" t="s">
+        <v>1146</v>
+      </c>
+    </row>
+    <row r="24" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>38</v>
       </c>
@@ -6112,8 +6184,11 @@
       <c r="P24" t="s">
         <v>1359</v>
       </c>
-    </row>
-    <row r="25" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="Q24" t="s">
+        <v>1147</v>
+      </c>
+    </row>
+    <row r="25" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>39</v>
       </c>
@@ -6157,8 +6232,11 @@
       <c r="P25" t="s">
         <v>1359</v>
       </c>
-    </row>
-    <row r="26" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="Q25" t="s">
+        <v>1165</v>
+      </c>
+    </row>
+    <row r="26" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>40</v>
       </c>
@@ -6202,8 +6280,11 @@
       <c r="P26" t="s">
         <v>1359</v>
       </c>
-    </row>
-    <row r="27" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="Q26" t="s">
+        <v>1166</v>
+      </c>
+    </row>
+    <row r="27" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>41</v>
       </c>
@@ -6247,8 +6328,11 @@
       <c r="P27" t="s">
         <v>1359</v>
       </c>
-    </row>
-    <row r="28" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="Q27" t="s">
+        <v>1167</v>
+      </c>
+    </row>
+    <row r="28" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>42</v>
       </c>
@@ -6292,8 +6376,11 @@
       <c r="P28" t="s">
         <v>1359</v>
       </c>
-    </row>
-    <row r="29" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="Q28" t="s">
+        <v>1168</v>
+      </c>
+    </row>
+    <row r="29" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>43</v>
       </c>
@@ -6337,8 +6424,11 @@
       <c r="P29" t="s">
         <v>1359</v>
       </c>
-    </row>
-    <row r="30" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="Q29" t="s">
+        <v>1169</v>
+      </c>
+    </row>
+    <row r="30" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>44</v>
       </c>
@@ -6382,8 +6472,11 @@
       <c r="P30" t="s">
         <v>1359</v>
       </c>
-    </row>
-    <row r="31" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="Q30" t="s">
+        <v>1169</v>
+      </c>
+    </row>
+    <row r="31" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>45</v>
       </c>
@@ -6424,8 +6517,11 @@
       <c r="P31" t="s">
         <v>1359</v>
       </c>
-    </row>
-    <row r="32" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="Q31" t="s">
+        <v>1194</v>
+      </c>
+    </row>
+    <row r="32" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>46</v>
       </c>
@@ -6466,8 +6562,11 @@
       <c r="P32" t="s">
         <v>1359</v>
       </c>
-    </row>
-    <row r="33" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="Q32" t="s">
+        <v>1195</v>
+      </c>
+    </row>
+    <row r="33" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>47</v>
       </c>
@@ -6508,8 +6607,11 @@
       <c r="P33" t="s">
         <v>1359</v>
       </c>
-    </row>
-    <row r="34" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="Q33" t="s">
+        <v>1196</v>
+      </c>
+    </row>
+    <row r="34" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>48</v>
       </c>
@@ -6550,8 +6652,11 @@
       <c r="P34" t="s">
         <v>1359</v>
       </c>
-    </row>
-    <row r="35" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="Q34" t="s">
+        <v>1197</v>
+      </c>
+    </row>
+    <row r="35" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>49</v>
       </c>
@@ -6592,8 +6697,11 @@
       <c r="P35" t="s">
         <v>1359</v>
       </c>
-    </row>
-    <row r="36" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="Q35" t="s">
+        <v>1198</v>
+      </c>
+    </row>
+    <row r="36" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>50</v>
       </c>
@@ -6631,8 +6739,11 @@
       <c r="P36" t="s">
         <v>1359</v>
       </c>
-    </row>
-    <row r="37" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="Q36" t="s">
+        <v>1199</v>
+      </c>
+    </row>
+    <row r="37" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>51</v>
       </c>
@@ -6673,8 +6784,11 @@
       <c r="P37" t="s">
         <v>1359</v>
       </c>
-    </row>
-    <row r="38" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="Q37" t="s">
+        <v>1200</v>
+      </c>
+    </row>
+    <row r="38" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>52</v>
       </c>
@@ -6715,8 +6829,11 @@
       <c r="P38" t="s">
         <v>1359</v>
       </c>
-    </row>
-    <row r="39" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="Q38" t="s">
+        <v>1201</v>
+      </c>
+    </row>
+    <row r="39" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>53</v>
       </c>
@@ -6760,8 +6877,11 @@
       <c r="P39" t="s">
         <v>1359</v>
       </c>
-    </row>
-    <row r="40" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="Q39" t="s">
+        <v>1222</v>
+      </c>
+    </row>
+    <row r="40" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>54</v>
       </c>
@@ -6805,8 +6925,11 @@
       <c r="P40" t="s">
         <v>1359</v>
       </c>
-    </row>
-    <row r="41" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="Q40" t="s">
+        <v>1223</v>
+      </c>
+    </row>
+    <row r="41" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>55</v>
       </c>
@@ -6850,8 +6973,11 @@
       <c r="P41" t="s">
         <v>1359</v>
       </c>
-    </row>
-    <row r="42" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="Q41" t="s">
+        <v>1224</v>
+      </c>
+    </row>
+    <row r="42" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>56</v>
       </c>
@@ -6895,8 +7021,11 @@
       <c r="P42" t="s">
         <v>1359</v>
       </c>
-    </row>
-    <row r="43" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="Q42" t="s">
+        <v>1225</v>
+      </c>
+    </row>
+    <row r="43" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>57</v>
       </c>
@@ -6940,8 +7069,11 @@
       <c r="P43" t="s">
         <v>1359</v>
       </c>
-    </row>
-    <row r="44" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="Q43" t="s">
+        <v>1226</v>
+      </c>
+    </row>
+    <row r="44" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>58</v>
       </c>
@@ -6985,8 +7117,11 @@
       <c r="P44" t="s">
         <v>1359</v>
       </c>
-    </row>
-    <row r="45" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="Q44" t="s">
+        <v>1240</v>
+      </c>
+    </row>
+    <row r="45" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>59</v>
       </c>
@@ -7030,8 +7165,11 @@
       <c r="P45" t="s">
         <v>1359</v>
       </c>
-    </row>
-    <row r="46" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="Q45" t="s">
+        <v>1241</v>
+      </c>
+    </row>
+    <row r="46" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>60</v>
       </c>
@@ -7075,8 +7213,11 @@
       <c r="P46" t="s">
         <v>1359</v>
       </c>
-    </row>
-    <row r="47" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="Q46" t="s">
+        <v>1242</v>
+      </c>
+    </row>
+    <row r="47" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
         <v>61</v>
       </c>
@@ -7120,8 +7261,11 @@
       <c r="P47" t="s">
         <v>1359</v>
       </c>
-    </row>
-    <row r="48" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="Q47" t="s">
+        <v>1243</v>
+      </c>
+    </row>
+    <row r="48" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
         <v>62</v>
       </c>
@@ -7165,8 +7309,11 @@
       <c r="P48" t="s">
         <v>1359</v>
       </c>
-    </row>
-    <row r="49" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="Q48" t="s">
+        <v>1244</v>
+      </c>
+    </row>
+    <row r="49" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
         <v>63</v>
       </c>
@@ -7210,8 +7357,11 @@
       <c r="P49" t="s">
         <v>1359</v>
       </c>
-    </row>
-    <row r="50" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="Q49" t="s">
+        <v>1257</v>
+      </c>
+    </row>
+    <row r="50" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
         <v>64</v>
       </c>
@@ -7255,8 +7405,11 @@
       <c r="P50" t="s">
         <v>1359</v>
       </c>
-    </row>
-    <row r="51" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="Q50" t="s">
+        <v>1258</v>
+      </c>
+    </row>
+    <row r="51" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
         <v>65</v>
       </c>
@@ -7300,8 +7453,11 @@
       <c r="P51" t="s">
         <v>1359</v>
       </c>
-    </row>
-    <row r="52" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="Q51" t="s">
+        <v>1259</v>
+      </c>
+    </row>
+    <row r="52" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
         <v>66</v>
       </c>
@@ -7345,8 +7501,11 @@
       <c r="P52" t="s">
         <v>1359</v>
       </c>
-    </row>
-    <row r="53" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="Q52" t="s">
+        <v>1260</v>
+      </c>
+    </row>
+    <row r="53" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
         <v>67</v>
       </c>
@@ -7390,8 +7549,11 @@
       <c r="P53" t="s">
         <v>1359</v>
       </c>
-    </row>
-    <row r="54" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="Q53" t="s">
+        <v>1261</v>
+      </c>
+    </row>
+    <row r="54" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
         <v>68</v>
       </c>
@@ -7435,8 +7597,11 @@
       <c r="P54" t="s">
         <v>1359</v>
       </c>
-    </row>
-    <row r="55" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="Q54" t="s">
+        <v>1262</v>
+      </c>
+    </row>
+    <row r="55" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
         <v>69</v>
       </c>
@@ -7480,8 +7645,11 @@
       <c r="P55" t="s">
         <v>1359</v>
       </c>
-    </row>
-    <row r="56" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="Q55" t="s">
+        <v>1281</v>
+      </c>
+    </row>
+    <row r="56" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
         <v>70</v>
       </c>
@@ -7525,8 +7693,11 @@
       <c r="P56" t="s">
         <v>1359</v>
       </c>
-    </row>
-    <row r="57" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="Q56" t="s">
+        <v>1285</v>
+      </c>
+    </row>
+    <row r="57" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
         <v>71</v>
       </c>
@@ -7570,8 +7741,11 @@
       <c r="P57" t="s">
         <v>1359</v>
       </c>
-    </row>
-    <row r="58" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="Q57" t="s">
+        <v>1289</v>
+      </c>
+    </row>
+    <row r="58" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
         <v>72</v>
       </c>
@@ -7615,8 +7789,11 @@
       <c r="P58" t="s">
         <v>1359</v>
       </c>
-    </row>
-    <row r="59" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="Q58" t="s">
+        <v>1294</v>
+      </c>
+    </row>
+    <row r="59" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
         <v>73</v>
       </c>
@@ -7660,8 +7837,11 @@
       <c r="P59" t="s">
         <v>1359</v>
       </c>
-    </row>
-    <row r="60" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="Q59" t="s">
+        <v>1297</v>
+      </c>
+    </row>
+    <row r="60" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
         <v>74</v>
       </c>
@@ -7705,8 +7885,11 @@
       <c r="P60" t="s">
         <v>1359</v>
       </c>
-    </row>
-    <row r="61" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="Q60" t="s">
+        <v>1298</v>
+      </c>
+    </row>
+    <row r="61" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
         <v>75</v>
       </c>
@@ -7750,8 +7933,11 @@
       <c r="P61" t="s">
         <v>1359</v>
       </c>
-    </row>
-    <row r="62" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="Q61" t="s">
+        <v>1299</v>
+      </c>
+    </row>
+    <row r="62" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
         <v>76</v>
       </c>
@@ -7795,8 +7981,11 @@
       <c r="P62" t="s">
         <v>1359</v>
       </c>
-    </row>
-    <row r="63" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="Q62" t="s">
+        <v>1300</v>
+      </c>
+    </row>
+    <row r="63" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
         <v>77</v>
       </c>
@@ -7840,8 +8029,11 @@
       <c r="P63" t="s">
         <v>1359</v>
       </c>
-    </row>
-    <row r="64" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="Q63" t="s">
+        <v>1301</v>
+      </c>
+    </row>
+    <row r="64" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
         <v>78</v>
       </c>
@@ -7885,8 +8077,11 @@
       <c r="P64" t="s">
         <v>1359</v>
       </c>
-    </row>
-    <row r="65" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="Q64" t="s">
+        <v>1302</v>
+      </c>
+    </row>
+    <row r="65" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
         <v>79</v>
       </c>
@@ -7930,8 +8125,11 @@
       <c r="P65" t="s">
         <v>1359</v>
       </c>
-    </row>
-    <row r="66" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="Q65" t="s">
+        <v>1303</v>
+      </c>
+    </row>
+    <row r="66" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
         <v>80</v>
       </c>
@@ -7975,8 +8173,11 @@
       <c r="P66" t="s">
         <v>1359</v>
       </c>
-    </row>
-    <row r="67" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="Q66" t="s">
+        <v>1304</v>
+      </c>
+    </row>
+    <row r="67" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
         <v>81</v>
       </c>
@@ -8020,8 +8221,11 @@
       <c r="P67" t="s">
         <v>1359</v>
       </c>
-    </row>
-    <row r="68" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="Q67" t="s">
+        <v>1305</v>
+      </c>
+    </row>
+    <row r="68" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
         <v>82</v>
       </c>
@@ -8065,8 +8269,11 @@
       <c r="P68" t="s">
         <v>1359</v>
       </c>
-    </row>
-    <row r="69" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="Q68" t="s">
+        <v>1306</v>
+      </c>
+    </row>
+    <row r="69" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
         <v>83</v>
       </c>
@@ -8110,8 +8317,11 @@
       <c r="P69" t="s">
         <v>1359</v>
       </c>
-    </row>
-    <row r="70" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="Q69" t="s">
+        <v>1331</v>
+      </c>
+    </row>
+    <row r="70" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
         <v>84</v>
       </c>
@@ -8155,8 +8365,11 @@
       <c r="P70" t="s">
         <v>1359</v>
       </c>
-    </row>
-    <row r="71" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="Q70" t="s">
+        <v>1332</v>
+      </c>
+    </row>
+    <row r="71" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
         <v>85</v>
       </c>
@@ -8200,8 +8413,11 @@
       <c r="P71" t="s">
         <v>1359</v>
       </c>
-    </row>
-    <row r="72" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="Q71" t="s">
+        <v>1333</v>
+      </c>
+    </row>
+    <row r="72" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
         <v>86</v>
       </c>
@@ -8245,8 +8461,11 @@
       <c r="P72" t="s">
         <v>1359</v>
       </c>
-    </row>
-    <row r="73" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="Q72" t="s">
+        <v>1338</v>
+      </c>
+    </row>
+    <row r="73" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
         <v>87</v>
       </c>
@@ -8290,8 +8509,11 @@
       <c r="P73" t="s">
         <v>1359</v>
       </c>
-    </row>
-    <row r="74" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="Q73" t="s">
+        <v>1341</v>
+      </c>
+    </row>
+    <row r="74" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
         <v>88</v>
       </c>
@@ -8335,8 +8557,11 @@
       <c r="P74" t="s">
         <v>1359</v>
       </c>
-    </row>
-    <row r="75" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="Q74" t="s">
+        <v>1342</v>
+      </c>
+    </row>
+    <row r="75" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
         <v>89</v>
       </c>
@@ -8380,8 +8605,11 @@
       <c r="P75" t="s">
         <v>1359</v>
       </c>
-    </row>
-    <row r="76" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="Q75" t="s">
+        <v>1343</v>
+      </c>
+    </row>
+    <row r="76" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
         <v>90</v>
       </c>
@@ -8425,8 +8653,11 @@
       <c r="P76" t="s">
         <v>1359</v>
       </c>
-    </row>
-    <row r="77" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="Q76" t="s">
+        <v>1349</v>
+      </c>
+    </row>
+    <row r="77" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
         <v>91</v>
       </c>
@@ -8470,8 +8701,11 @@
       <c r="P77" t="s">
         <v>1359</v>
       </c>
-    </row>
-    <row r="78" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="Q77" t="s">
+        <v>1352</v>
+      </c>
+    </row>
+    <row r="78" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
         <v>92</v>
       </c>
@@ -8515,8 +8749,11 @@
       <c r="P78" t="s">
         <v>1359</v>
       </c>
-    </row>
-    <row r="79" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="Q78" t="s">
+        <v>1360</v>
+      </c>
+    </row>
+    <row r="79" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
         <v>93</v>
       </c>
@@ -8560,8 +8797,11 @@
       <c r="P79" t="s">
         <v>1359</v>
       </c>
-    </row>
-    <row r="80" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="Q79" t="s">
+        <v>1364</v>
+      </c>
+    </row>
+    <row r="80" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
         <v>94</v>
       </c>
@@ -8608,8 +8848,11 @@
       <c r="P80" t="s">
         <v>1359</v>
       </c>
-    </row>
-    <row r="81" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="Q80" t="s">
+        <v>1365</v>
+      </c>
+    </row>
+    <row r="81" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
         <v>95</v>
       </c>
@@ -8656,8 +8899,11 @@
       <c r="P81" t="s">
         <v>1359</v>
       </c>
-    </row>
-    <row r="82" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="Q81" t="s">
+        <v>1366</v>
+      </c>
+    </row>
+    <row r="82" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
         <v>96</v>
       </c>
@@ -8704,8 +8950,11 @@
       <c r="P82" t="s">
         <v>1359</v>
       </c>
-    </row>
-    <row r="83" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="Q82" t="s">
+        <v>1367</v>
+      </c>
+    </row>
+    <row r="83" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
         <v>97</v>
       </c>
@@ -8752,8 +9001,11 @@
       <c r="P83" t="s">
         <v>1359</v>
       </c>
-    </row>
-    <row r="84" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="Q83" t="s">
+        <v>1376</v>
+      </c>
+    </row>
+    <row r="84" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
         <v>98</v>
       </c>
@@ -8800,8 +9052,11 @@
       <c r="P84" t="s">
         <v>1359</v>
       </c>
-    </row>
-    <row r="85" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="Q84" t="s">
+        <v>1377</v>
+      </c>
+    </row>
+    <row r="85" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
         <v>99</v>
       </c>
@@ -8848,8 +9103,11 @@
       <c r="P85" t="s">
         <v>1359</v>
       </c>
-    </row>
-    <row r="86" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="Q85" t="s">
+        <v>1378</v>
+      </c>
+    </row>
+    <row r="86" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
         <v>100</v>
       </c>
@@ -8896,8 +9154,11 @@
       <c r="P86" t="s">
         <v>1359</v>
       </c>
-    </row>
-    <row r="87" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="Q86" t="s">
+        <v>1379</v>
+      </c>
+    </row>
+    <row r="87" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
         <v>101</v>
       </c>
@@ -8944,8 +9205,11 @@
       <c r="P87" t="s">
         <v>1359</v>
       </c>
-    </row>
-    <row r="88" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="Q87" t="s">
+        <v>1380</v>
+      </c>
+    </row>
+    <row r="88" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
         <v>102</v>
       </c>
@@ -8992,8 +9256,11 @@
       <c r="P88" t="s">
         <v>1359</v>
       </c>
-    </row>
-    <row r="89" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="Q88" t="s">
+        <v>1381</v>
+      </c>
+    </row>
+    <row r="89" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
         <v>103</v>
       </c>
@@ -9037,8 +9304,11 @@
       <c r="P89" t="s">
         <v>1359</v>
       </c>
-    </row>
-    <row r="90" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="Q89" t="s">
+        <v>1398</v>
+      </c>
+    </row>
+    <row r="90" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A90" t="s">
         <v>104</v>
       </c>
@@ -9085,8 +9355,11 @@
       <c r="P90" t="s">
         <v>1359</v>
       </c>
-    </row>
-    <row r="91" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="Q90" t="s">
+        <v>1401</v>
+      </c>
+    </row>
+    <row r="91" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A91" t="s">
         <v>105</v>
       </c>
@@ -9133,8 +9406,11 @@
       <c r="P91" t="s">
         <v>1359</v>
       </c>
-    </row>
-    <row r="92" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="Q91" t="s">
+        <v>1402</v>
+      </c>
+    </row>
+    <row r="92" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A92" t="s">
         <v>106</v>
       </c>
@@ -9181,8 +9457,11 @@
       <c r="P92" t="s">
         <v>1359</v>
       </c>
-    </row>
-    <row r="93" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="Q92" t="s">
+        <v>1403</v>
+      </c>
+    </row>
+    <row r="93" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A93" t="s">
         <v>107</v>
       </c>
@@ -9229,8 +9508,11 @@
       <c r="P93" t="s">
         <v>1359</v>
       </c>
-    </row>
-    <row r="94" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="Q93" t="s">
+        <v>1404</v>
+      </c>
+    </row>
+    <row r="94" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A94" t="s">
         <v>108</v>
       </c>
@@ -9277,8 +9559,11 @@
       <c r="P94" t="s">
         <v>1359</v>
       </c>
-    </row>
-    <row r="95" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="Q94" t="s">
+        <v>1411</v>
+      </c>
+    </row>
+    <row r="95" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A95" t="s">
         <v>109</v>
       </c>
@@ -9325,8 +9610,11 @@
       <c r="P95" t="s">
         <v>1359</v>
       </c>
-    </row>
-    <row r="96" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="Q95" t="s">
+        <v>1412</v>
+      </c>
+    </row>
+    <row r="96" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A96" t="s">
         <v>110</v>
       </c>
@@ -9370,8 +9658,11 @@
       <c r="P96" t="s">
         <v>1359</v>
       </c>
-    </row>
-    <row r="97" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="Q96" t="s">
+        <v>1419</v>
+      </c>
+    </row>
+    <row r="97" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A97" t="s">
         <v>111</v>
       </c>
@@ -9415,8 +9706,11 @@
       <c r="P97" t="s">
         <v>1359</v>
       </c>
-    </row>
-    <row r="98" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="Q97" t="s">
+        <v>1423</v>
+      </c>
+    </row>
+    <row r="98" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A98" t="s">
         <v>112</v>
       </c>
@@ -9442,7 +9736,7 @@
         <v>1164</v>
       </c>
       <c r="I98" t="s">
-        <v>1434</v>
+        <v>1531</v>
       </c>
       <c r="J98">
         <v>4300</v>
@@ -9463,13 +9757,16 @@
       <c r="P98" t="s">
         <v>1359</v>
       </c>
-    </row>
-    <row r="99" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="Q98" t="s">
+        <v>1433</v>
+      </c>
+    </row>
+    <row r="99" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A99" t="s">
         <v>113</v>
       </c>
       <c r="B99" t="s">
-        <v>1441</v>
+        <v>1435</v>
       </c>
       <c r="C99" t="s">
         <v>1426</v>
@@ -9481,7 +9778,7 @@
         <v>1074</v>
       </c>
       <c r="F99" t="s">
-        <v>1440</v>
+        <v>1434</v>
       </c>
       <c r="G99" t="s">
         <v>1428</v>
@@ -9490,7 +9787,7 @@
         <v>1164</v>
       </c>
       <c r="I99" t="s">
-        <v>1435</v>
+        <v>1532</v>
       </c>
       <c r="J99">
         <v>4300</v>
@@ -9511,13 +9808,16 @@
       <c r="P99" t="s">
         <v>1359</v>
       </c>
-    </row>
-    <row r="100" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="Q99" t="s">
+        <v>1435</v>
+      </c>
+    </row>
+    <row r="100" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A100" t="s">
         <v>114</v>
       </c>
       <c r="B100" t="s">
-        <v>1442</v>
+        <v>1436</v>
       </c>
       <c r="C100" t="s">
         <v>1426</v>
@@ -9529,7 +9829,7 @@
         <v>1074</v>
       </c>
       <c r="F100" t="s">
-        <v>1440</v>
+        <v>1434</v>
       </c>
       <c r="G100" t="s">
         <v>1429</v>
@@ -9538,7 +9838,7 @@
         <v>1164</v>
       </c>
       <c r="I100" t="s">
-        <v>1436</v>
+        <v>1533</v>
       </c>
       <c r="J100">
         <v>4300</v>
@@ -9559,13 +9859,16 @@
       <c r="P100" t="s">
         <v>1359</v>
       </c>
-    </row>
-    <row r="101" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="Q100" t="s">
+        <v>1436</v>
+      </c>
+    </row>
+    <row r="101" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A101" t="s">
         <v>115</v>
       </c>
       <c r="B101" t="s">
-        <v>1443</v>
+        <v>1437</v>
       </c>
       <c r="C101" t="s">
         <v>1426</v>
@@ -9577,7 +9880,7 @@
         <v>1074</v>
       </c>
       <c r="F101" t="s">
-        <v>1440</v>
+        <v>1434</v>
       </c>
       <c r="G101" t="s">
         <v>1430</v>
@@ -9586,7 +9889,7 @@
         <v>1164</v>
       </c>
       <c r="I101" t="s">
-        <v>1437</v>
+        <v>1534</v>
       </c>
       <c r="J101">
         <v>4300</v>
@@ -9607,13 +9910,16 @@
       <c r="P101" t="s">
         <v>1359</v>
       </c>
-    </row>
-    <row r="102" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="Q101" t="s">
+        <v>1437</v>
+      </c>
+    </row>
+    <row r="102" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A102" t="s">
         <v>116</v>
       </c>
       <c r="B102" t="s">
-        <v>1444</v>
+        <v>1438</v>
       </c>
       <c r="C102" t="s">
         <v>1426</v>
@@ -9625,7 +9931,7 @@
         <v>1074</v>
       </c>
       <c r="F102" t="s">
-        <v>1440</v>
+        <v>1434</v>
       </c>
       <c r="G102" t="s">
         <v>1431</v>
@@ -9634,7 +9940,7 @@
         <v>1164</v>
       </c>
       <c r="I102" t="s">
-        <v>1438</v>
+        <v>1535</v>
       </c>
       <c r="J102">
         <v>4300</v>
@@ -9655,13 +9961,16 @@
       <c r="P102" t="s">
         <v>1359</v>
       </c>
-    </row>
-    <row r="103" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="Q102" t="s">
+        <v>1438</v>
+      </c>
+    </row>
+    <row r="103" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A103" t="s">
         <v>117</v>
       </c>
       <c r="B103" t="s">
-        <v>1445</v>
+        <v>1439</v>
       </c>
       <c r="C103" t="s">
         <v>1426</v>
@@ -9673,7 +9982,7 @@
         <v>1074</v>
       </c>
       <c r="F103" t="s">
-        <v>1440</v>
+        <v>1434</v>
       </c>
       <c r="G103" t="s">
         <v>1432</v>
@@ -9682,7 +9991,7 @@
         <v>1164</v>
       </c>
       <c r="I103" t="s">
-        <v>1439</v>
+        <v>1536</v>
       </c>
       <c r="J103">
         <v>4300</v>
@@ -9703,34 +10012,37 @@
       <c r="P103" t="s">
         <v>1359</v>
       </c>
-    </row>
-    <row r="104" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="Q103" t="s">
+        <v>1439</v>
+      </c>
+    </row>
+    <row r="104" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A104" t="s">
         <v>118</v>
       </c>
       <c r="B104" t="s">
-        <v>1446</v>
+        <v>1440</v>
       </c>
       <c r="C104" t="s">
-        <v>1460</v>
+        <v>1454</v>
       </c>
       <c r="D104" t="s">
-        <v>1462</v>
+        <v>1456</v>
       </c>
       <c r="E104" t="s">
-        <v>1461</v>
+        <v>1455</v>
       </c>
       <c r="F104" t="s">
-        <v>1462</v>
+        <v>1456</v>
       </c>
       <c r="G104" t="s">
-        <v>1463</v>
+        <v>1457</v>
       </c>
       <c r="H104" t="s">
         <v>1164</v>
       </c>
       <c r="I104" t="s">
-        <v>1475</v>
+        <v>1469</v>
       </c>
       <c r="J104">
         <v>1600</v>
@@ -9751,34 +10063,37 @@
       <c r="P104" t="s">
         <v>1359</v>
       </c>
-    </row>
-    <row r="105" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="Q104" t="s">
+        <v>1440</v>
+      </c>
+    </row>
+    <row r="105" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A105" t="s">
         <v>119</v>
       </c>
       <c r="B105" t="s">
-        <v>1447</v>
+        <v>1441</v>
       </c>
       <c r="C105" t="s">
-        <v>1460</v>
+        <v>1454</v>
       </c>
       <c r="D105" t="s">
-        <v>1462</v>
+        <v>1456</v>
       </c>
       <c r="E105" t="s">
-        <v>1461</v>
+        <v>1455</v>
       </c>
       <c r="F105" t="s">
-        <v>1462</v>
+        <v>1456</v>
       </c>
       <c r="G105" t="s">
-        <v>1464</v>
+        <v>1458</v>
       </c>
       <c r="H105" t="s">
         <v>1164</v>
       </c>
       <c r="I105" t="s">
-        <v>1476</v>
+        <v>1470</v>
       </c>
       <c r="J105">
         <v>1600</v>
@@ -9799,25 +10114,28 @@
       <c r="P105" t="s">
         <v>1359</v>
       </c>
-    </row>
-    <row r="106" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="Q105" t="s">
+        <v>1441</v>
+      </c>
+    </row>
+    <row r="106" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A106" t="s">
         <v>120</v>
       </c>
       <c r="B106" t="s">
-        <v>1448</v>
+        <v>1442</v>
       </c>
       <c r="C106" t="s">
-        <v>1460</v>
+        <v>1454</v>
       </c>
       <c r="D106" t="s">
-        <v>1462</v>
+        <v>1456</v>
       </c>
       <c r="E106" t="s">
-        <v>1461</v>
+        <v>1455</v>
       </c>
       <c r="F106" t="s">
-        <v>1462</v>
+        <v>1456</v>
       </c>
       <c r="G106" t="s">
         <v>1431</v>
@@ -9826,7 +10144,7 @@
         <v>1164</v>
       </c>
       <c r="I106" t="s">
-        <v>1477</v>
+        <v>1471</v>
       </c>
       <c r="J106">
         <v>1600</v>
@@ -9847,34 +10165,37 @@
       <c r="P106" t="s">
         <v>1359</v>
       </c>
-    </row>
-    <row r="107" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="Q106" t="s">
+        <v>1442</v>
+      </c>
+    </row>
+    <row r="107" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A107" t="s">
         <v>121</v>
       </c>
       <c r="B107" t="s">
-        <v>1449</v>
+        <v>1443</v>
       </c>
       <c r="C107" t="s">
-        <v>1460</v>
+        <v>1454</v>
       </c>
       <c r="D107" t="s">
-        <v>1462</v>
+        <v>1456</v>
       </c>
       <c r="E107" t="s">
-        <v>1461</v>
+        <v>1455</v>
       </c>
       <c r="F107" t="s">
-        <v>1462</v>
+        <v>1456</v>
       </c>
       <c r="G107" t="s">
-        <v>1465</v>
+        <v>1459</v>
       </c>
       <c r="H107" t="s">
         <v>1164</v>
       </c>
       <c r="I107" t="s">
-        <v>1478</v>
+        <v>1472</v>
       </c>
       <c r="J107">
         <v>1600</v>
@@ -9895,25 +10216,28 @@
       <c r="P107" t="s">
         <v>1359</v>
       </c>
-    </row>
-    <row r="108" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="Q107" t="s">
+        <v>1443</v>
+      </c>
+    </row>
+    <row r="108" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A108" t="s">
         <v>122</v>
       </c>
       <c r="B108" t="s">
-        <v>1450</v>
+        <v>1444</v>
       </c>
       <c r="C108" t="s">
-        <v>1460</v>
+        <v>1454</v>
       </c>
       <c r="D108" t="s">
-        <v>1462</v>
+        <v>1456</v>
       </c>
       <c r="E108" t="s">
-        <v>1461</v>
+        <v>1455</v>
       </c>
       <c r="F108" t="s">
-        <v>1462</v>
+        <v>1456</v>
       </c>
       <c r="G108" t="s">
         <v>1429</v>
@@ -9922,7 +10246,7 @@
         <v>1164</v>
       </c>
       <c r="I108" t="s">
-        <v>1479</v>
+        <v>1473</v>
       </c>
       <c r="J108">
         <v>1600</v>
@@ -9943,34 +10267,37 @@
       <c r="P108" t="s">
         <v>1359</v>
       </c>
-    </row>
-    <row r="109" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="Q108" t="s">
+        <v>1444</v>
+      </c>
+    </row>
+    <row r="109" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A109" t="s">
         <v>123</v>
       </c>
       <c r="B109" t="s">
-        <v>1451</v>
+        <v>1445</v>
       </c>
       <c r="C109" t="s">
+        <v>1454</v>
+      </c>
+      <c r="D109" t="s">
+        <v>1456</v>
+      </c>
+      <c r="E109" t="s">
+        <v>1455</v>
+      </c>
+      <c r="F109" t="s">
+        <v>1456</v>
+      </c>
+      <c r="G109" t="s">
         <v>1460</v>
-      </c>
-      <c r="D109" t="s">
-        <v>1462</v>
-      </c>
-      <c r="E109" t="s">
-        <v>1461</v>
-      </c>
-      <c r="F109" t="s">
-        <v>1462</v>
-      </c>
-      <c r="G109" t="s">
-        <v>1466</v>
       </c>
       <c r="H109" t="s">
         <v>1164</v>
       </c>
       <c r="I109" t="s">
-        <v>1480</v>
+        <v>1474</v>
       </c>
       <c r="J109">
         <v>1600</v>
@@ -9991,34 +10318,37 @@
       <c r="P109" t="s">
         <v>1359</v>
       </c>
-    </row>
-    <row r="110" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="Q109" t="s">
+        <v>1445</v>
+      </c>
+    </row>
+    <row r="110" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A110" t="s">
         <v>124</v>
       </c>
       <c r="B110" t="s">
-        <v>1452</v>
+        <v>1446</v>
       </c>
       <c r="C110" t="s">
-        <v>1460</v>
+        <v>1454</v>
       </c>
       <c r="D110" t="s">
-        <v>1462</v>
+        <v>1456</v>
       </c>
       <c r="E110" t="s">
+        <v>1455</v>
+      </c>
+      <c r="F110" t="s">
+        <v>1456</v>
+      </c>
+      <c r="G110" t="s">
         <v>1461</v>
-      </c>
-      <c r="F110" t="s">
-        <v>1462</v>
-      </c>
-      <c r="G110" t="s">
-        <v>1467</v>
       </c>
       <c r="H110" t="s">
         <v>1164</v>
       </c>
       <c r="I110" t="s">
-        <v>1481</v>
+        <v>1475</v>
       </c>
       <c r="J110">
         <v>1600</v>
@@ -10039,34 +10369,37 @@
       <c r="P110" t="s">
         <v>1359</v>
       </c>
-    </row>
-    <row r="111" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="Q110" t="s">
+        <v>1446</v>
+      </c>
+    </row>
+    <row r="111" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A111" t="s">
         <v>125</v>
       </c>
       <c r="B111" t="s">
-        <v>1453</v>
+        <v>1447</v>
       </c>
       <c r="C111" t="s">
-        <v>1460</v>
+        <v>1454</v>
       </c>
       <c r="D111" t="s">
+        <v>1456</v>
+      </c>
+      <c r="E111" t="s">
+        <v>1455</v>
+      </c>
+      <c r="F111" t="s">
+        <v>1456</v>
+      </c>
+      <c r="G111" t="s">
         <v>1462</v>
-      </c>
-      <c r="E111" t="s">
-        <v>1461</v>
-      </c>
-      <c r="F111" t="s">
-        <v>1462</v>
-      </c>
-      <c r="G111" t="s">
-        <v>1468</v>
       </c>
       <c r="H111" t="s">
         <v>1164</v>
       </c>
       <c r="I111" t="s">
-        <v>1482</v>
+        <v>1476</v>
       </c>
       <c r="J111">
         <v>1600</v>
@@ -10087,34 +10420,37 @@
       <c r="P111" t="s">
         <v>1359</v>
       </c>
-    </row>
-    <row r="112" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="Q111" t="s">
+        <v>1447</v>
+      </c>
+    </row>
+    <row r="112" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A112" t="s">
         <v>126</v>
       </c>
       <c r="B112" t="s">
+        <v>1448</v>
+      </c>
+      <c r="C112" t="s">
         <v>1454</v>
       </c>
-      <c r="C112" t="s">
-        <v>1460</v>
-      </c>
       <c r="D112" t="s">
-        <v>1462</v>
+        <v>1456</v>
       </c>
       <c r="E112" t="s">
-        <v>1461</v>
+        <v>1455</v>
       </c>
       <c r="F112" t="s">
-        <v>1462</v>
+        <v>1456</v>
       </c>
       <c r="G112" t="s">
-        <v>1469</v>
+        <v>1463</v>
       </c>
       <c r="H112" t="s">
         <v>1164</v>
       </c>
       <c r="I112" t="s">
-        <v>1483</v>
+        <v>1477</v>
       </c>
       <c r="J112">
         <v>1600</v>
@@ -10135,34 +10471,37 @@
       <c r="P112" t="s">
         <v>1359</v>
       </c>
-    </row>
-    <row r="113" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="Q112" t="s">
+        <v>1448</v>
+      </c>
+    </row>
+    <row r="113" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A113" t="s">
         <v>127</v>
       </c>
       <c r="B113" t="s">
+        <v>1449</v>
+      </c>
+      <c r="C113" t="s">
+        <v>1454</v>
+      </c>
+      <c r="D113" t="s">
+        <v>1456</v>
+      </c>
+      <c r="E113" t="s">
         <v>1455</v>
       </c>
-      <c r="C113" t="s">
-        <v>1460</v>
-      </c>
-      <c r="D113" t="s">
-        <v>1462</v>
-      </c>
-      <c r="E113" t="s">
-        <v>1461</v>
-      </c>
       <c r="F113" t="s">
-        <v>1462</v>
+        <v>1456</v>
       </c>
       <c r="G113" t="s">
-        <v>1470</v>
+        <v>1464</v>
       </c>
       <c r="H113" t="s">
         <v>1164</v>
       </c>
       <c r="I113" t="s">
-        <v>1484</v>
+        <v>1478</v>
       </c>
       <c r="J113">
         <v>1600</v>
@@ -10183,34 +10522,37 @@
       <c r="P113" t="s">
         <v>1359</v>
       </c>
-    </row>
-    <row r="114" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="Q113" t="s">
+        <v>1449</v>
+      </c>
+    </row>
+    <row r="114" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A114" t="s">
         <v>128</v>
       </c>
       <c r="B114" t="s">
+        <v>1450</v>
+      </c>
+      <c r="C114" t="s">
+        <v>1454</v>
+      </c>
+      <c r="D114" t="s">
         <v>1456</v>
       </c>
-      <c r="C114" t="s">
-        <v>1460</v>
-      </c>
-      <c r="D114" t="s">
-        <v>1462</v>
-      </c>
       <c r="E114" t="s">
-        <v>1461</v>
+        <v>1455</v>
       </c>
       <c r="F114" t="s">
-        <v>1462</v>
+        <v>1456</v>
       </c>
       <c r="G114" t="s">
-        <v>1471</v>
+        <v>1465</v>
       </c>
       <c r="H114" t="s">
         <v>1164</v>
       </c>
       <c r="I114" t="s">
-        <v>1485</v>
+        <v>1479</v>
       </c>
       <c r="J114">
         <v>1600</v>
@@ -10231,34 +10573,37 @@
       <c r="P114" t="s">
         <v>1359</v>
       </c>
-    </row>
-    <row r="115" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="Q114" t="s">
+        <v>1450</v>
+      </c>
+    </row>
+    <row r="115" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A115" t="s">
         <v>129</v>
       </c>
       <c r="B115" t="s">
-        <v>1457</v>
+        <v>1451</v>
       </c>
       <c r="C115" t="s">
-        <v>1460</v>
+        <v>1454</v>
       </c>
       <c r="D115" t="s">
-        <v>1462</v>
+        <v>1456</v>
       </c>
       <c r="E115" t="s">
-        <v>1461</v>
+        <v>1455</v>
       </c>
       <c r="F115" t="s">
-        <v>1462</v>
+        <v>1456</v>
       </c>
       <c r="G115" t="s">
-        <v>1472</v>
+        <v>1466</v>
       </c>
       <c r="H115" t="s">
         <v>1164</v>
       </c>
       <c r="I115" t="s">
-        <v>1486</v>
+        <v>1480</v>
       </c>
       <c r="J115">
         <v>1600</v>
@@ -10279,34 +10624,37 @@
       <c r="P115" t="s">
         <v>1359</v>
       </c>
-    </row>
-    <row r="116" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="Q115" t="s">
+        <v>1451</v>
+      </c>
+    </row>
+    <row r="116" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A116" t="s">
         <v>130</v>
       </c>
       <c r="B116" t="s">
-        <v>1458</v>
+        <v>1452</v>
       </c>
       <c r="C116" t="s">
-        <v>1460</v>
+        <v>1454</v>
       </c>
       <c r="D116" t="s">
-        <v>1462</v>
+        <v>1456</v>
       </c>
       <c r="E116" t="s">
-        <v>1461</v>
+        <v>1455</v>
       </c>
       <c r="F116" t="s">
-        <v>1462</v>
+        <v>1456</v>
       </c>
       <c r="G116" t="s">
-        <v>1473</v>
+        <v>1467</v>
       </c>
       <c r="H116" t="s">
         <v>1164</v>
       </c>
       <c r="I116" t="s">
-        <v>1487</v>
+        <v>1481</v>
       </c>
       <c r="J116">
         <v>1600</v>
@@ -10327,34 +10675,37 @@
       <c r="P116" t="s">
         <v>1359</v>
       </c>
-    </row>
-    <row r="117" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="Q116" t="s">
+        <v>1452</v>
+      </c>
+    </row>
+    <row r="117" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A117" t="s">
         <v>131</v>
       </c>
       <c r="B117" t="s">
-        <v>1459</v>
+        <v>1453</v>
       </c>
       <c r="C117" t="s">
-        <v>1460</v>
+        <v>1454</v>
       </c>
       <c r="D117" t="s">
-        <v>1462</v>
+        <v>1456</v>
       </c>
       <c r="E117" t="s">
-        <v>1461</v>
+        <v>1455</v>
       </c>
       <c r="F117" t="s">
-        <v>1462</v>
+        <v>1456</v>
       </c>
       <c r="G117" t="s">
-        <v>1474</v>
+        <v>1468</v>
       </c>
       <c r="H117" t="s">
         <v>1164</v>
       </c>
       <c r="I117" t="s">
-        <v>1488</v>
+        <v>1482</v>
       </c>
       <c r="J117">
         <v>1600</v>
@@ -10375,34 +10726,37 @@
       <c r="P117" t="s">
         <v>1359</v>
       </c>
-    </row>
-    <row r="118" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="Q117" t="s">
+        <v>1453</v>
+      </c>
+    </row>
+    <row r="118" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A118" t="s">
         <v>132</v>
       </c>
       <c r="B118" t="s">
-        <v>1489</v>
+        <v>1483</v>
       </c>
       <c r="C118" t="s">
-        <v>1460</v>
+        <v>1454</v>
       </c>
       <c r="D118" t="s">
-        <v>1497</v>
+        <v>1491</v>
       </c>
       <c r="E118" t="s">
-        <v>1461</v>
+        <v>1455</v>
       </c>
       <c r="F118" t="s">
-        <v>1497</v>
+        <v>1491</v>
       </c>
       <c r="G118" t="s">
-        <v>1463</v>
+        <v>1457</v>
       </c>
       <c r="H118" t="s">
         <v>1164</v>
       </c>
       <c r="I118" t="s">
-        <v>1502</v>
+        <v>1496</v>
       </c>
       <c r="J118">
         <v>2000</v>
@@ -10423,34 +10777,37 @@
       <c r="P118" t="s">
         <v>1359</v>
       </c>
-    </row>
-    <row r="119" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="Q118" t="s">
+        <v>1483</v>
+      </c>
+    </row>
+    <row r="119" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A119" t="s">
         <v>133</v>
       </c>
       <c r="B119" t="s">
-        <v>1490</v>
+        <v>1484</v>
       </c>
       <c r="C119" t="s">
-        <v>1460</v>
+        <v>1454</v>
       </c>
       <c r="D119" t="s">
-        <v>1497</v>
+        <v>1491</v>
       </c>
       <c r="E119" t="s">
-        <v>1461</v>
+        <v>1455</v>
       </c>
       <c r="F119" t="s">
-        <v>1497</v>
+        <v>1491</v>
       </c>
       <c r="G119" t="s">
-        <v>1464</v>
+        <v>1458</v>
       </c>
       <c r="H119" t="s">
         <v>1164</v>
       </c>
       <c r="I119" t="s">
-        <v>1503</v>
+        <v>1497</v>
       </c>
       <c r="J119">
         <v>2000</v>
@@ -10471,34 +10828,37 @@
       <c r="P119" t="s">
         <v>1359</v>
       </c>
-    </row>
-    <row r="120" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="Q119" t="s">
+        <v>1484</v>
+      </c>
+    </row>
+    <row r="120" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A120" t="s">
         <v>134</v>
       </c>
       <c r="B120" t="s">
+        <v>1485</v>
+      </c>
+      <c r="C120" t="s">
+        <v>1454</v>
+      </c>
+      <c r="D120" t="s">
         <v>1491</v>
       </c>
-      <c r="C120" t="s">
-        <v>1460</v>
-      </c>
-      <c r="D120" t="s">
-        <v>1497</v>
-      </c>
       <c r="E120" t="s">
+        <v>1455</v>
+      </c>
+      <c r="F120" t="s">
+        <v>1491</v>
+      </c>
+      <c r="G120" t="s">
         <v>1461</v>
-      </c>
-      <c r="F120" t="s">
-        <v>1497</v>
-      </c>
-      <c r="G120" t="s">
-        <v>1467</v>
       </c>
       <c r="H120" t="s">
         <v>1164</v>
       </c>
       <c r="I120" t="s">
-        <v>1504</v>
+        <v>1498</v>
       </c>
       <c r="J120">
         <v>2000</v>
@@ -10519,34 +10879,37 @@
       <c r="P120" t="s">
         <v>1359</v>
       </c>
-    </row>
-    <row r="121" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="Q120" t="s">
+        <v>1485</v>
+      </c>
+    </row>
+    <row r="121" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A121" t="s">
         <v>135</v>
       </c>
       <c r="B121" t="s">
+        <v>1486</v>
+      </c>
+      <c r="C121" t="s">
+        <v>1454</v>
+      </c>
+      <c r="D121" t="s">
+        <v>1491</v>
+      </c>
+      <c r="E121" t="s">
+        <v>1455</v>
+      </c>
+      <c r="F121" t="s">
+        <v>1491</v>
+      </c>
+      <c r="G121" t="s">
         <v>1492</v>
-      </c>
-      <c r="C121" t="s">
-        <v>1460</v>
-      </c>
-      <c r="D121" t="s">
-        <v>1497</v>
-      </c>
-      <c r="E121" t="s">
-        <v>1461</v>
-      </c>
-      <c r="F121" t="s">
-        <v>1497</v>
-      </c>
-      <c r="G121" t="s">
-        <v>1498</v>
       </c>
       <c r="H121" t="s">
         <v>1164</v>
       </c>
       <c r="I121" t="s">
-        <v>1505</v>
+        <v>1499</v>
       </c>
       <c r="J121">
         <v>2000</v>
@@ -10567,34 +10930,37 @@
       <c r="P121" t="s">
         <v>1359</v>
       </c>
-    </row>
-    <row r="122" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="Q121" t="s">
+        <v>1486</v>
+      </c>
+    </row>
+    <row r="122" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A122" t="s">
         <v>136</v>
       </c>
       <c r="B122" t="s">
+        <v>1487</v>
+      </c>
+      <c r="C122" t="s">
+        <v>1454</v>
+      </c>
+      <c r="D122" t="s">
+        <v>1491</v>
+      </c>
+      <c r="E122" t="s">
+        <v>1455</v>
+      </c>
+      <c r="F122" t="s">
+        <v>1491</v>
+      </c>
+      <c r="G122" t="s">
         <v>1493</v>
-      </c>
-      <c r="C122" t="s">
-        <v>1460</v>
-      </c>
-      <c r="D122" t="s">
-        <v>1497</v>
-      </c>
-      <c r="E122" t="s">
-        <v>1461</v>
-      </c>
-      <c r="F122" t="s">
-        <v>1497</v>
-      </c>
-      <c r="G122" t="s">
-        <v>1499</v>
       </c>
       <c r="H122" t="s">
         <v>1164</v>
       </c>
       <c r="I122" t="s">
-        <v>1506</v>
+        <v>1500</v>
       </c>
       <c r="J122">
         <v>2000</v>
@@ -10615,34 +10981,37 @@
       <c r="P122" t="s">
         <v>1359</v>
       </c>
-    </row>
-    <row r="123" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="Q122" t="s">
+        <v>1487</v>
+      </c>
+    </row>
+    <row r="123" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A123" t="s">
         <v>137</v>
       </c>
       <c r="B123" t="s">
+        <v>1488</v>
+      </c>
+      <c r="C123" t="s">
+        <v>1454</v>
+      </c>
+      <c r="D123" t="s">
+        <v>1491</v>
+      </c>
+      <c r="E123" t="s">
+        <v>1455</v>
+      </c>
+      <c r="F123" t="s">
+        <v>1491</v>
+      </c>
+      <c r="G123" t="s">
         <v>1494</v>
-      </c>
-      <c r="C123" t="s">
-        <v>1460</v>
-      </c>
-      <c r="D123" t="s">
-        <v>1497</v>
-      </c>
-      <c r="E123" t="s">
-        <v>1461</v>
-      </c>
-      <c r="F123" t="s">
-        <v>1497</v>
-      </c>
-      <c r="G123" t="s">
-        <v>1500</v>
       </c>
       <c r="H123" t="s">
         <v>1164</v>
       </c>
       <c r="I123" t="s">
-        <v>1507</v>
+        <v>1501</v>
       </c>
       <c r="J123">
         <v>2000</v>
@@ -10663,34 +11032,37 @@
       <c r="P123" t="s">
         <v>1359</v>
       </c>
-    </row>
-    <row r="124" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="Q123" t="s">
+        <v>1488</v>
+      </c>
+    </row>
+    <row r="124" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A124" t="s">
         <v>138</v>
       </c>
       <c r="B124" t="s">
-        <v>1495</v>
+        <v>1489</v>
       </c>
       <c r="C124" t="s">
-        <v>1460</v>
+        <v>1454</v>
       </c>
       <c r="D124" t="s">
-        <v>1497</v>
+        <v>1491</v>
       </c>
       <c r="E124" t="s">
-        <v>1461</v>
+        <v>1455</v>
       </c>
       <c r="F124" t="s">
-        <v>1497</v>
+        <v>1491</v>
       </c>
       <c r="G124" t="s">
-        <v>1465</v>
+        <v>1459</v>
       </c>
       <c r="H124" t="s">
         <v>1164</v>
       </c>
       <c r="I124" t="s">
-        <v>1508</v>
+        <v>1502</v>
       </c>
       <c r="J124">
         <v>2000</v>
@@ -10711,34 +11083,37 @@
       <c r="P124" t="s">
         <v>1359</v>
       </c>
-    </row>
-    <row r="125" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="Q124" t="s">
+        <v>1489</v>
+      </c>
+    </row>
+    <row r="125" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A125" t="s">
         <v>139</v>
       </c>
       <c r="B125" t="s">
-        <v>1496</v>
+        <v>1490</v>
       </c>
       <c r="C125" t="s">
-        <v>1460</v>
+        <v>1454</v>
       </c>
       <c r="D125" t="s">
-        <v>1497</v>
+        <v>1491</v>
       </c>
       <c r="E125" t="s">
-        <v>1461</v>
+        <v>1455</v>
       </c>
       <c r="F125" t="s">
-        <v>1497</v>
+        <v>1491</v>
       </c>
       <c r="G125" t="s">
-        <v>1501</v>
+        <v>1495</v>
       </c>
       <c r="H125" t="s">
         <v>1164</v>
       </c>
       <c r="I125" t="s">
-        <v>1509</v>
+        <v>1503</v>
       </c>
       <c r="J125">
         <v>2000</v>
@@ -10759,34 +11134,37 @@
       <c r="P125" t="s">
         <v>1359</v>
       </c>
-    </row>
-    <row r="126" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="Q125" t="s">
+        <v>1490</v>
+      </c>
+    </row>
+    <row r="126" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A126" t="s">
         <v>140</v>
       </c>
       <c r="B126" t="s">
+        <v>1504</v>
+      </c>
+      <c r="C126" t="s">
+        <v>1454</v>
+      </c>
+      <c r="D126" t="s">
+        <v>1509</v>
+      </c>
+      <c r="E126" t="s">
+        <v>1455</v>
+      </c>
+      <c r="F126" t="s">
+        <v>1509</v>
+      </c>
+      <c r="G126" t="s">
         <v>1510</v>
-      </c>
-      <c r="C126" t="s">
-        <v>1460</v>
-      </c>
-      <c r="D126" t="s">
-        <v>1515</v>
-      </c>
-      <c r="E126" t="s">
-        <v>1461</v>
-      </c>
-      <c r="F126" t="s">
-        <v>1515</v>
-      </c>
-      <c r="G126" t="s">
-        <v>1516</v>
       </c>
       <c r="H126" t="s">
         <v>1164</v>
       </c>
       <c r="I126" t="s">
-        <v>1521</v>
+        <v>1515</v>
       </c>
       <c r="J126">
         <v>2000</v>
@@ -10807,34 +11185,37 @@
       <c r="P126" t="s">
         <v>1359</v>
       </c>
-    </row>
-    <row r="127" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="Q126" t="s">
+        <v>1504</v>
+      </c>
+    </row>
+    <row r="127" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A127" t="s">
         <v>141</v>
       </c>
       <c r="B127" t="s">
+        <v>1505</v>
+      </c>
+      <c r="C127" t="s">
+        <v>1454</v>
+      </c>
+      <c r="D127" t="s">
+        <v>1509</v>
+      </c>
+      <c r="E127" t="s">
+        <v>1455</v>
+      </c>
+      <c r="F127" t="s">
+        <v>1509</v>
+      </c>
+      <c r="G127" t="s">
         <v>1511</v>
-      </c>
-      <c r="C127" t="s">
-        <v>1460</v>
-      </c>
-      <c r="D127" t="s">
-        <v>1515</v>
-      </c>
-      <c r="E127" t="s">
-        <v>1461</v>
-      </c>
-      <c r="F127" t="s">
-        <v>1515</v>
-      </c>
-      <c r="G127" t="s">
-        <v>1517</v>
       </c>
       <c r="H127" t="s">
         <v>1164</v>
       </c>
       <c r="I127" t="s">
-        <v>1522</v>
+        <v>1516</v>
       </c>
       <c r="J127">
         <v>2000</v>
@@ -10855,34 +11236,37 @@
       <c r="P127" t="s">
         <v>1359</v>
       </c>
-    </row>
-    <row r="128" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="Q127" t="s">
+        <v>1505</v>
+      </c>
+    </row>
+    <row r="128" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A128" t="s">
         <v>142</v>
       </c>
       <c r="B128" t="s">
+        <v>1506</v>
+      </c>
+      <c r="C128" t="s">
+        <v>1454</v>
+      </c>
+      <c r="D128" t="s">
+        <v>1509</v>
+      </c>
+      <c r="E128" t="s">
+        <v>1455</v>
+      </c>
+      <c r="F128" t="s">
+        <v>1509</v>
+      </c>
+      <c r="G128" t="s">
         <v>1512</v>
-      </c>
-      <c r="C128" t="s">
-        <v>1460</v>
-      </c>
-      <c r="D128" t="s">
-        <v>1515</v>
-      </c>
-      <c r="E128" t="s">
-        <v>1461</v>
-      </c>
-      <c r="F128" t="s">
-        <v>1515</v>
-      </c>
-      <c r="G128" t="s">
-        <v>1518</v>
       </c>
       <c r="H128" t="s">
         <v>1164</v>
       </c>
       <c r="I128" t="s">
-        <v>1523</v>
+        <v>1517</v>
       </c>
       <c r="J128">
         <v>2000</v>
@@ -10903,34 +11287,37 @@
       <c r="P128" t="s">
         <v>1359</v>
       </c>
-    </row>
-    <row r="129" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="Q128" t="s">
+        <v>1506</v>
+      </c>
+    </row>
+    <row r="129" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A129" t="s">
         <v>143</v>
       </c>
       <c r="B129" t="s">
+        <v>1507</v>
+      </c>
+      <c r="C129" t="s">
+        <v>1454</v>
+      </c>
+      <c r="D129" t="s">
+        <v>1509</v>
+      </c>
+      <c r="E129" t="s">
+        <v>1455</v>
+      </c>
+      <c r="F129" t="s">
+        <v>1509</v>
+      </c>
+      <c r="G129" t="s">
         <v>1513</v>
-      </c>
-      <c r="C129" t="s">
-        <v>1460</v>
-      </c>
-      <c r="D129" t="s">
-        <v>1515</v>
-      </c>
-      <c r="E129" t="s">
-        <v>1461</v>
-      </c>
-      <c r="F129" t="s">
-        <v>1515</v>
-      </c>
-      <c r="G129" t="s">
-        <v>1519</v>
       </c>
       <c r="H129" t="s">
         <v>1164</v>
       </c>
       <c r="I129" t="s">
-        <v>1524</v>
+        <v>1518</v>
       </c>
       <c r="J129">
         <v>2000</v>
@@ -10951,34 +11338,37 @@
       <c r="P129" t="s">
         <v>1359</v>
       </c>
-    </row>
-    <row r="130" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="Q129" t="s">
+        <v>1507</v>
+      </c>
+    </row>
+    <row r="130" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A130" t="s">
         <v>144</v>
       </c>
       <c r="B130" t="s">
+        <v>1508</v>
+      </c>
+      <c r="C130" t="s">
+        <v>1454</v>
+      </c>
+      <c r="D130" t="s">
+        <v>1509</v>
+      </c>
+      <c r="E130" t="s">
+        <v>1455</v>
+      </c>
+      <c r="F130" t="s">
+        <v>1509</v>
+      </c>
+      <c r="G130" t="s">
         <v>1514</v>
-      </c>
-      <c r="C130" t="s">
-        <v>1460</v>
-      </c>
-      <c r="D130" t="s">
-        <v>1515</v>
-      </c>
-      <c r="E130" t="s">
-        <v>1461</v>
-      </c>
-      <c r="F130" t="s">
-        <v>1515</v>
-      </c>
-      <c r="G130" t="s">
-        <v>1520</v>
       </c>
       <c r="H130" t="s">
         <v>1164</v>
       </c>
       <c r="I130" t="s">
-        <v>1525</v>
+        <v>1519</v>
       </c>
       <c r="J130">
         <v>2000</v>
@@ -10999,31 +11389,34 @@
       <c r="P130" t="s">
         <v>1359</v>
       </c>
-    </row>
-    <row r="131" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="Q130" t="s">
+        <v>1508</v>
+      </c>
+    </row>
+    <row r="131" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A131" t="s">
         <v>145</v>
       </c>
       <c r="B131" t="s">
-        <v>1526</v>
+        <v>1520</v>
       </c>
       <c r="C131" t="s">
-        <v>1529</v>
+        <v>1523</v>
       </c>
       <c r="D131" t="s">
-        <v>1530</v>
+        <v>1524</v>
       </c>
       <c r="E131" t="s">
         <v>1074</v>
       </c>
       <c r="F131" t="s">
-        <v>1530</v>
+        <v>1524</v>
       </c>
       <c r="H131" t="s">
         <v>1164</v>
       </c>
       <c r="I131" t="s">
-        <v>1534</v>
+        <v>1528</v>
       </c>
       <c r="J131">
         <v>20000</v>
@@ -11044,31 +11437,34 @@
       <c r="P131" t="s">
         <v>1358</v>
       </c>
-    </row>
-    <row r="132" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="Q131" t="s">
+        <v>1520</v>
+      </c>
+    </row>
+    <row r="132" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A132" t="s">
         <v>146</v>
       </c>
       <c r="B132" t="s">
-        <v>1527</v>
+        <v>1521</v>
       </c>
       <c r="C132" t="s">
-        <v>1529</v>
+        <v>1523</v>
       </c>
       <c r="D132" t="s">
-        <v>1531</v>
+        <v>1525</v>
       </c>
       <c r="E132" t="s">
         <v>1074</v>
       </c>
       <c r="F132" t="s">
-        <v>1532</v>
+        <v>1526</v>
       </c>
       <c r="H132" t="s">
         <v>1164</v>
       </c>
       <c r="I132" t="s">
-        <v>1535</v>
+        <v>1529</v>
       </c>
       <c r="J132">
         <v>6500</v>
@@ -11089,31 +11485,34 @@
       <c r="P132" t="s">
         <v>1358</v>
       </c>
-    </row>
-    <row r="133" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="Q132" t="s">
+        <v>1521</v>
+      </c>
+    </row>
+    <row r="133" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A133" t="s">
         <v>147</v>
       </c>
       <c r="B133" t="s">
-        <v>1528</v>
+        <v>1522</v>
       </c>
       <c r="C133" t="s">
-        <v>1529</v>
+        <v>1523</v>
       </c>
       <c r="D133" t="s">
-        <v>1533</v>
+        <v>1527</v>
       </c>
       <c r="E133" t="s">
         <v>1074</v>
       </c>
       <c r="F133" t="s">
-        <v>1533</v>
+        <v>1527</v>
       </c>
       <c r="H133" t="s">
         <v>1164</v>
       </c>
       <c r="I133" t="s">
-        <v>1536</v>
+        <v>1530</v>
       </c>
       <c r="J133">
         <v>9000</v>
@@ -11134,8 +11533,11 @@
       <c r="P133" t="s">
         <v>1358</v>
       </c>
-    </row>
-    <row r="134" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="Q133" t="s">
+        <v>1522</v>
+      </c>
+    </row>
+    <row r="134" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A134" t="s">
         <v>148</v>
       </c>
@@ -11156,7 +11558,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="135" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="135" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A135" t="s">
         <v>149</v>
       </c>
@@ -11177,7 +11579,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="136" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="136" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A136" t="s">
         <v>150</v>
       </c>
@@ -11198,7 +11600,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="137" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="137" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A137" t="s">
         <v>151</v>
       </c>
@@ -11219,7 +11621,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="138" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="138" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A138" t="s">
         <v>152</v>
       </c>
@@ -11240,7 +11642,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="139" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="139" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A139" t="s">
         <v>153</v>
       </c>
@@ -11261,7 +11663,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="140" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="140" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A140" t="s">
         <v>154</v>
       </c>
@@ -11282,7 +11684,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="141" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="141" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A141" t="s">
         <v>155</v>
       </c>
@@ -11303,7 +11705,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="142" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="142" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A142" t="s">
         <v>156</v>
       </c>
@@ -11324,7 +11726,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="143" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="143" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A143" t="s">
         <v>157</v>
       </c>
@@ -11345,7 +11747,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="144" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="144" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A144" t="s">
         <v>158</v>
       </c>

</xml_diff>